<commit_message>
feat(rebuild): two-gate system, all-sport collectors, training scripts, audit deliverables
</commit_message>
<xml_diff>
--- a/data/flat/mlb.xlsx
+++ b/data/flat/mlb.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Picks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Picks" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Summary'!$A$1:$L$19</definedName>
@@ -57790,12 +57790,12 @@
     <row r="186" ht="36" customHeight="1">
       <c r="A186" s="24" t="inlineStr">
         <is>
-          <t>6ff3540567964bef</t>
+          <t>5f545bf126614044</t>
         </is>
       </c>
       <c r="B186" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C186" s="24" t="inlineStr">
@@ -57840,20 +57840,20 @@
         </is>
       </c>
       <c r="L186" s="26" t="n">
-        <v>-156</v>
+        <v>-174</v>
       </c>
       <c r="M186" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.574713</v>
       </c>
       <c r="N186" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.635036</v>
       </c>
       <c r="O186" s="28" t="n">
         <v>0.543314</v>
       </c>
       <c r="P186" s="28" t="n"/>
       <c r="Q186" s="28" t="n">
-        <v>-0.06606099999999999</v>
+        <v>-0.091722</v>
       </c>
       <c r="R186" s="26" t="n">
         <v>0</v>
@@ -57882,7 +57882,7 @@
       <c r="AD186" s="24" t="n"/>
       <c r="AE186" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.6100 (aec-mlb-tor-hou-2026-08-05); model edge vs ask -0.0667.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.6350 (aec-mlb-tor-hou-2026-08-05); model edge vs ask -0.0917.</t>
         </is>
       </c>
       <c r="AF186" s="31" t="inlineStr">
@@ -58001,7 +58001,7 @@
       </c>
       <c r="BH186" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:50.122845Z</t>
+          <t>2026-08-05T13:52:24.506232Z</t>
         </is>
       </c>
       <c r="BI186" s="24" t="inlineStr">
@@ -58011,16 +58011,16 @@
       </c>
       <c r="BJ186" s="25" t="n"/>
       <c r="BK186" s="26" t="n">
-        <v>-156</v>
+        <v>-174</v>
       </c>
       <c r="BL186" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.574713</v>
       </c>
       <c r="BM186" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.635036</v>
       </c>
       <c r="BN186" s="28" t="n">
-        <v>0.606965</v>
+        <v>0.631841</v>
       </c>
       <c r="BO186" s="28" t="n"/>
       <c r="BP186" s="25" t="n"/>
@@ -58093,12 +58093,12 @@
     <row r="187" ht="36" customHeight="1">
       <c r="A187" s="24" t="inlineStr">
         <is>
-          <t>7bfbbb9e10304374</t>
+          <t>2533a73a6e144c45</t>
         </is>
       </c>
       <c r="B187" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C187" s="24" t="inlineStr">
@@ -58152,11 +58152,11 @@
         <v>0.534884</v>
       </c>
       <c r="O187" s="28" t="n">
-        <v>0.522292</v>
+        <v>0.522352</v>
       </c>
       <c r="P187" s="28" t="n"/>
       <c r="Q187" s="28" t="n">
-        <v>-0.012592</v>
+        <v>-0.012532</v>
       </c>
       <c r="R187" s="26" t="n">
         <v>15</v>
@@ -58185,7 +58185,7 @@
       <c r="AD187" s="24" t="n"/>
       <c r="AE187" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5350 (aec-mlb-lad-chc-2026-08-05); model edge vs ask -0.0127.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5350 (aec-mlb-lad-chc-2026-08-05); model edge vs ask -0.0126.</t>
         </is>
       </c>
       <c r="AF187" s="31" t="inlineStr">
@@ -58289,7 +58289,7 @@
       </c>
       <c r="BE187" s="24" t="inlineStr">
         <is>
-          <t>cd121ba990e73d6d</t>
+          <t>7d69706ac5e95086</t>
         </is>
       </c>
       <c r="BF187" s="24" t="inlineStr">
@@ -58304,7 +58304,7 @@
       </c>
       <c r="BH187" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:50.628303Z</t>
+          <t>2026-08-05T13:52:24.994220Z</t>
         </is>
       </c>
       <c r="BI187" s="24" t="inlineStr">
@@ -58356,7 +58356,7 @@
       </c>
       <c r="CF187" s="24" t="inlineStr">
         <is>
-          <t>1.0097</t>
+          <t>1.0089</t>
         </is>
       </c>
       <c r="CG187" s="24" t="n"/>
@@ -58384,7 +58384,7 @@
       <c r="CQ187" s="24" t="n"/>
       <c r="CR187" s="24" t="inlineStr">
         <is>
-          <t>0.522292</t>
+          <t>0.522352</t>
         </is>
       </c>
       <c r="CS187" s="24" t="inlineStr">
@@ -58396,12 +58396,12 @@
     <row r="188" ht="36" customHeight="1">
       <c r="A188" s="24" t="inlineStr">
         <is>
-          <t>213b1d6df73b46a3</t>
+          <t>ae2fc2d9c7c44ae0</t>
         </is>
       </c>
       <c r="B188" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C188" s="24" t="inlineStr">
@@ -58446,23 +58446,23 @@
         </is>
       </c>
       <c r="L188" s="26" t="n">
-        <v>-167</v>
+        <v>-163</v>
       </c>
       <c r="M188" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.613497</v>
       </c>
       <c r="N188" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.619772</v>
       </c>
       <c r="O188" s="28" t="n">
         <v>0.585182</v>
       </c>
       <c r="P188" s="28" t="n"/>
       <c r="Q188" s="28" t="n">
-        <v>-0.040286</v>
+        <v>-0.03459</v>
       </c>
       <c r="R188" s="26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="S188" s="29" t="n">
         <v>0</v>
@@ -58488,7 +58488,7 @@
       <c r="AD188" s="24" t="n"/>
       <c r="AE188" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.6250 (aec-mlb-sf-tex-2026-08-05); model edge vs ask -0.0398.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.6200 (aec-mlb-sf-tex-2026-08-05); model edge vs ask -0.0348.</t>
         </is>
       </c>
       <c r="AF188" s="31" t="inlineStr">
@@ -58607,7 +58607,7 @@
       </c>
       <c r="BH188" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:51.533440Z</t>
+          <t>2026-08-05T13:52:25.614756Z</t>
         </is>
       </c>
       <c r="BI188" s="24" t="inlineStr">
@@ -58617,16 +58617,16 @@
       </c>
       <c r="BJ188" s="25" t="n"/>
       <c r="BK188" s="26" t="n">
-        <v>-167</v>
+        <v>-163</v>
       </c>
       <c r="BL188" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.613497</v>
       </c>
       <c r="BM188" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.619772</v>
       </c>
       <c r="BN188" s="28" t="n">
-        <v>0.621891</v>
+        <v>0.616915</v>
       </c>
       <c r="BO188" s="28" t="n"/>
       <c r="BP188" s="25" t="n"/>
@@ -58699,12 +58699,12 @@
     <row r="189" ht="36" customHeight="1">
       <c r="A189" s="24" t="inlineStr">
         <is>
-          <t>1ecfa20ee3cd46f5</t>
+          <t>51149c5ad9e34fb7</t>
         </is>
       </c>
       <c r="B189" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C189" s="24" t="inlineStr">
@@ -58749,23 +58749,23 @@
         </is>
       </c>
       <c r="L189" s="26" t="n">
-        <v>-147</v>
+        <v>-153</v>
       </c>
       <c r="M189" s="27" t="n">
-        <v>1.680272</v>
+        <v>1.653595</v>
       </c>
       <c r="N189" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.604743</v>
       </c>
       <c r="O189" s="28" t="n">
-        <v>0.651419</v>
+        <v>0.651358</v>
       </c>
       <c r="P189" s="28" t="n"/>
       <c r="Q189" s="28" t="n">
-        <v>0.056277</v>
+        <v>0.046615</v>
       </c>
       <c r="R189" s="26" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="S189" s="29" t="n">
         <v>1.75</v>
@@ -58791,7 +58791,7 @@
       <c r="AD189" s="24" t="n"/>
       <c r="AE189" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5950 (aec-mlb-tb-col-2026-08-05); model edge vs ask +0.0564.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.6050 (aec-mlb-tb-col-2026-08-05); model edge vs ask +0.0464.</t>
         </is>
       </c>
       <c r="AF189" s="31" t="inlineStr">
@@ -58895,7 +58895,7 @@
       </c>
       <c r="BE189" s="24" t="inlineStr">
         <is>
-          <t>afbdfea2d660f7f9</t>
+          <t>133a0f8d2d67fce5</t>
         </is>
       </c>
       <c r="BF189" s="24" t="inlineStr">
@@ -58910,7 +58910,7 @@
       </c>
       <c r="BH189" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:52.558033Z</t>
+          <t>2026-08-05T13:52:26.086277Z</t>
         </is>
       </c>
       <c r="BI189" s="24" t="inlineStr">
@@ -58920,16 +58920,16 @@
       </c>
       <c r="BJ189" s="25" t="n"/>
       <c r="BK189" s="26" t="n">
-        <v>-147</v>
+        <v>-153</v>
       </c>
       <c r="BL189" s="27" t="n">
-        <v>1.680272</v>
+        <v>1.653595</v>
       </c>
       <c r="BM189" s="28" t="n">
-        <v>0.5951419999999999</v>
+        <v>0.604743</v>
       </c>
       <c r="BN189" s="28" t="n">
-        <v>0.59204</v>
+        <v>0.60199</v>
       </c>
       <c r="BO189" s="28" t="n"/>
       <c r="BP189" s="25" t="n"/>
@@ -58962,7 +58962,7 @@
       </c>
       <c r="CF189" s="24" t="inlineStr">
         <is>
-          <t>1.0105</t>
+          <t>1.0096</t>
         </is>
       </c>
       <c r="CG189" s="24" t="n"/>
@@ -58990,7 +58990,7 @@
       <c r="CQ189" s="24" t="n"/>
       <c r="CR189" s="24" t="inlineStr">
         <is>
-          <t>0.651419</t>
+          <t>0.651358</t>
         </is>
       </c>
       <c r="CS189" s="24" t="inlineStr">
@@ -59002,12 +59002,12 @@
     <row r="190" ht="36" customHeight="1">
       <c r="A190" s="24" t="inlineStr">
         <is>
-          <t>834fa6cfaa72498f</t>
+          <t>dc6ca6079a734a5f</t>
         </is>
       </c>
       <c r="B190" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C190" s="24" t="inlineStr">
@@ -59052,23 +59052,23 @@
         </is>
       </c>
       <c r="L190" s="26" t="n">
-        <v>-130</v>
+        <v>-117</v>
       </c>
       <c r="M190" s="27" t="n">
-        <v>1.769231</v>
+        <v>1.854701</v>
       </c>
       <c r="N190" s="28" t="n">
-        <v>0.565217</v>
+        <v>0.539171</v>
       </c>
       <c r="O190" s="28" t="n">
-        <v>0.620283</v>
+        <v>0.620156</v>
       </c>
       <c r="P190" s="28" t="n"/>
       <c r="Q190" s="28" t="n">
-        <v>0.055066</v>
+        <v>0.080985</v>
       </c>
       <c r="R190" s="26" t="n">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="S190" s="29" t="n">
         <v>1.5</v>
@@ -59094,7 +59094,7 @@
       <c r="AD190" s="24" t="n"/>
       <c r="AE190" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5650 (aec-mlb-laa-bal-2026-08-05); model edge vs ask +0.0553.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5400 (aec-mlb-laa-bal-2026-08-05); model edge vs ask +0.0802.</t>
         </is>
       </c>
       <c r="AF190" s="31" t="inlineStr">
@@ -59198,7 +59198,7 @@
       </c>
       <c r="BE190" s="24" t="inlineStr">
         <is>
-          <t>0c5ef877e6b12160</t>
+          <t>90250452b4135146</t>
         </is>
       </c>
       <c r="BF190" s="24" t="inlineStr">
@@ -59213,7 +59213,7 @@
       </c>
       <c r="BH190" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:53.451157Z</t>
+          <t>2026-08-05T13:52:26.546603Z</t>
         </is>
       </c>
       <c r="BI190" s="24" t="inlineStr">
@@ -59223,16 +59223,16 @@
       </c>
       <c r="BJ190" s="25" t="n"/>
       <c r="BK190" s="26" t="n">
-        <v>-130</v>
+        <v>-117</v>
       </c>
       <c r="BL190" s="27" t="n">
-        <v>1.769231</v>
+        <v>1.854701</v>
       </c>
       <c r="BM190" s="28" t="n">
-        <v>0.565217</v>
+        <v>0.539171</v>
       </c>
       <c r="BN190" s="28" t="n">
-        <v>0.562189</v>
+        <v>0.537313</v>
       </c>
       <c r="BO190" s="28" t="n"/>
       <c r="BP190" s="25" t="n"/>
@@ -59265,7 +59265,7 @@
       </c>
       <c r="CF190" s="24" t="inlineStr">
         <is>
-          <t>1.0102</t>
+          <t>1.012</t>
         </is>
       </c>
       <c r="CG190" s="24" t="n"/>
@@ -59293,7 +59293,7 @@
       <c r="CQ190" s="24" t="n"/>
       <c r="CR190" s="24" t="inlineStr">
         <is>
-          <t>0.620283</t>
+          <t>0.620156</t>
         </is>
       </c>
       <c r="CS190" s="24" t="inlineStr">
@@ -59305,12 +59305,12 @@
     <row r="191" ht="36" customHeight="1">
       <c r="A191" s="24" t="inlineStr">
         <is>
-          <t>b3c6b3cca4c3426f</t>
+          <t>e3a6b3fee6d14874</t>
         </is>
       </c>
       <c r="B191" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C191" s="24" t="inlineStr">
@@ -59355,23 +59355,23 @@
         </is>
       </c>
       <c r="L191" s="26" t="n">
-        <v>-127</v>
+        <v>-135</v>
       </c>
       <c r="M191" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.740741</v>
       </c>
       <c r="N191" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.574468</v>
       </c>
       <c r="O191" s="28" t="n">
-        <v>0.531988</v>
+        <v>0.531981</v>
       </c>
       <c r="P191" s="28" t="n"/>
       <c r="Q191" s="28" t="n">
-        <v>-0.027483</v>
+        <v>-0.042487</v>
       </c>
       <c r="R191" s="26" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="S191" s="29" t="n">
         <v>0</v>
@@ -59397,7 +59397,7 @@
       <c r="AD191" s="24" t="n"/>
       <c r="AE191" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5600 (aec-mlb-ath-cin-2026-08-05); model edge vs ask -0.0280.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5750 (aec-mlb-ath-cin-2026-08-05); model edge vs ask -0.0430.</t>
         </is>
       </c>
       <c r="AF191" s="31" t="inlineStr">
@@ -59501,7 +59501,7 @@
       </c>
       <c r="BE191" s="24" t="inlineStr">
         <is>
-          <t>117cc3945a0a3429</t>
+          <t>b37c86ce3baa60b2</t>
         </is>
       </c>
       <c r="BF191" s="24" t="inlineStr">
@@ -59516,7 +59516,7 @@
       </c>
       <c r="BH191" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:56.201811Z</t>
+          <t>2026-08-05T13:52:28.221956Z</t>
         </is>
       </c>
       <c r="BI191" s="24" t="inlineStr">
@@ -59526,16 +59526,16 @@
       </c>
       <c r="BJ191" s="25" t="n"/>
       <c r="BK191" s="26" t="n">
-        <v>-127</v>
+        <v>-135</v>
       </c>
       <c r="BL191" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.740741</v>
       </c>
       <c r="BM191" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.574468</v>
       </c>
       <c r="BN191" s="28" t="n">
-        <v>0.557214</v>
+        <v>0.572139</v>
       </c>
       <c r="BO191" s="28" t="n"/>
       <c r="BP191" s="25" t="n"/>
@@ -59568,7 +59568,7 @@
       </c>
       <c r="CF191" s="24" t="inlineStr">
         <is>
-          <t>1.0202</t>
+          <t>1.0203</t>
         </is>
       </c>
       <c r="CG191" s="24" t="n"/>
@@ -59596,7 +59596,7 @@
       <c r="CQ191" s="24" t="n"/>
       <c r="CR191" s="24" t="inlineStr">
         <is>
-          <t>0.531988</t>
+          <t>0.531981</t>
         </is>
       </c>
       <c r="CS191" s="24" t="inlineStr">
@@ -59608,12 +59608,12 @@
     <row r="192" ht="36" customHeight="1">
       <c r="A192" s="24" t="inlineStr">
         <is>
-          <t>ea183039e65241a5</t>
+          <t>2b50414866bd4838</t>
         </is>
       </c>
       <c r="B192" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C192" s="24" t="inlineStr">
@@ -59658,23 +59658,23 @@
         </is>
       </c>
       <c r="L192" s="26" t="n">
-        <v>106</v>
+        <v>-104</v>
       </c>
       <c r="M192" s="27" t="n">
-        <v>2.06</v>
+        <v>1.961538</v>
       </c>
       <c r="N192" s="28" t="n">
-        <v>0.485437</v>
+        <v>0.509804</v>
       </c>
       <c r="O192" s="28" t="n">
-        <v>0.570001</v>
+        <v>0.570059</v>
       </c>
       <c r="P192" s="28" t="n"/>
       <c r="Q192" s="28" t="n">
-        <v>0.084564</v>
+        <v>0.060255</v>
       </c>
       <c r="R192" s="26" t="n">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="S192" s="29" t="n">
         <v>0</v>
@@ -59700,7 +59700,7 @@
       <c r="AD192" s="24" t="n"/>
       <c r="AE192" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.4850 (aec-mlb-nym-cle-2026-08-05); model edge vs ask +0.0850.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5100 (aec-mlb-nym-cle-2026-08-05); model edge vs ask +0.0601.</t>
         </is>
       </c>
       <c r="AF192" s="31" t="inlineStr">
@@ -59804,7 +59804,7 @@
       </c>
       <c r="BE192" s="24" t="inlineStr">
         <is>
-          <t>e56570441b5f5cf2</t>
+          <t>a8496f0544fb49ff</t>
         </is>
       </c>
       <c r="BF192" s="24" t="inlineStr">
@@ -59819,7 +59819,7 @@
       </c>
       <c r="BH192" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:55.141566Z</t>
+          <t>2026-08-05T13:52:27.503942Z</t>
         </is>
       </c>
       <c r="BI192" s="24" t="inlineStr">
@@ -59829,16 +59829,16 @@
       </c>
       <c r="BJ192" s="25" t="n"/>
       <c r="BK192" s="26" t="n">
-        <v>106</v>
+        <v>-104</v>
       </c>
       <c r="BL192" s="27" t="n">
-        <v>2.06</v>
+        <v>1.961538</v>
       </c>
       <c r="BM192" s="28" t="n">
-        <v>0.485437</v>
+        <v>0.509804</v>
       </c>
       <c r="BN192" s="28" t="n">
-        <v>0.482587</v>
+        <v>0.507463</v>
       </c>
       <c r="BO192" s="28" t="n"/>
       <c r="BP192" s="25" t="n"/>
@@ -59871,7 +59871,7 @@
       </c>
       <c r="CF192" s="24" t="inlineStr">
         <is>
-          <t>1.0127</t>
+          <t>1.0119</t>
         </is>
       </c>
       <c r="CG192" s="24" t="n"/>
@@ -59899,7 +59899,7 @@
       <c r="CQ192" s="24" t="n"/>
       <c r="CR192" s="24" t="inlineStr">
         <is>
-          <t>0.570001</t>
+          <t>0.570059</t>
         </is>
       </c>
       <c r="CS192" s="24" t="inlineStr">
@@ -59911,12 +59911,12 @@
     <row r="193" ht="36" customHeight="1">
       <c r="A193" s="24" t="inlineStr">
         <is>
-          <t>554772c4dc254e8d</t>
+          <t>0707206819d14a7d</t>
         </is>
       </c>
       <c r="B193" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C193" s="24" t="inlineStr">
@@ -59961,20 +59961,20 @@
         </is>
       </c>
       <c r="L193" s="26" t="n">
-        <v>-160</v>
+        <v>-174</v>
       </c>
       <c r="M193" s="27" t="n">
-        <v>1.625</v>
+        <v>1.574713</v>
       </c>
       <c r="N193" s="28" t="n">
-        <v>0.615385</v>
+        <v>0.635036</v>
       </c>
       <c r="O193" s="28" t="n">
-        <v>0.568075</v>
+        <v>0.568112</v>
       </c>
       <c r="P193" s="28" t="n"/>
       <c r="Q193" s="28" t="n">
-        <v>-0.04731</v>
+        <v>-0.066924</v>
       </c>
       <c r="R193" s="26" t="n">
         <v>0</v>
@@ -60003,7 +60003,7 @@
       <c r="AD193" s="24" t="n"/>
       <c r="AE193" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.6150 (aec-mlb-wsh-phi-2026-08-05); model edge vs ask -0.0469.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.6350 (aec-mlb-wsh-phi-2026-08-05); model edge vs ask -0.0669.</t>
         </is>
       </c>
       <c r="AF193" s="31" t="inlineStr">
@@ -60107,7 +60107,7 @@
       </c>
       <c r="BE193" s="24" t="inlineStr">
         <is>
-          <t>cc0cc1936c4cd2d0</t>
+          <t>28c4190bf888aff9</t>
         </is>
       </c>
       <c r="BF193" s="24" t="inlineStr">
@@ -60122,7 +60122,7 @@
       </c>
       <c r="BH193" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:54.460834Z</t>
+          <t>2026-08-05T13:52:27.109583Z</t>
         </is>
       </c>
       <c r="BI193" s="24" t="inlineStr">
@@ -60132,16 +60132,16 @@
       </c>
       <c r="BJ193" s="25" t="n"/>
       <c r="BK193" s="26" t="n">
-        <v>-160</v>
+        <v>-174</v>
       </c>
       <c r="BL193" s="27" t="n">
-        <v>1.625</v>
+        <v>1.574713</v>
       </c>
       <c r="BM193" s="28" t="n">
-        <v>0.615385</v>
+        <v>0.635036</v>
       </c>
       <c r="BN193" s="28" t="n">
-        <v>0.61194</v>
+        <v>0.631841</v>
       </c>
       <c r="BO193" s="28" t="n"/>
       <c r="BP193" s="25" t="n"/>
@@ -60174,7 +60174,7 @@
       </c>
       <c r="CF193" s="24" t="inlineStr">
         <is>
-          <t>1.0112</t>
+          <t>1.0107</t>
         </is>
       </c>
       <c r="CG193" s="24" t="n"/>
@@ -60202,7 +60202,7 @@
       <c r="CQ193" s="24" t="n"/>
       <c r="CR193" s="24" t="inlineStr">
         <is>
-          <t>0.568075</t>
+          <t>0.568112</t>
         </is>
       </c>
       <c r="CS193" s="24" t="inlineStr">
@@ -60214,12 +60214,12 @@
     <row r="194" ht="36" customHeight="1">
       <c r="A194" s="24" t="inlineStr">
         <is>
-          <t>6173832403c34386</t>
+          <t>0e57b7e2b084476b</t>
         </is>
       </c>
       <c r="B194" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C194" s="24" t="inlineStr">
@@ -60273,11 +60273,11 @@
         <v>0.590164</v>
       </c>
       <c r="O194" s="28" t="n">
-        <v>0.585723</v>
+        <v>0.5858100000000001</v>
       </c>
       <c r="P194" s="28" t="n"/>
       <c r="Q194" s="28" t="n">
-        <v>-0.004441</v>
+        <v>-0.004354</v>
       </c>
       <c r="R194" s="26" t="n">
         <v>19</v>
@@ -60306,7 +60306,7 @@
       <c r="AD194" s="24" t="n"/>
       <c r="AE194" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5900 (aec-mlb-stl-nyy-2026-08-05); model edge vs ask -0.0043.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5900 (aec-mlb-stl-nyy-2026-08-05); model edge vs ask -0.0042.</t>
         </is>
       </c>
       <c r="AF194" s="31" t="inlineStr">
@@ -60410,7 +60410,7 @@
       </c>
       <c r="BE194" s="24" t="inlineStr">
         <is>
-          <t>5e4023ab8bd19cc5</t>
+          <t>f16100c8dde61330</t>
         </is>
       </c>
       <c r="BF194" s="24" t="inlineStr">
@@ -60425,7 +60425,7 @@
       </c>
       <c r="BH194" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:57.037353Z</t>
+          <t>2026-08-05T13:52:28.745980Z</t>
         </is>
       </c>
       <c r="BI194" s="24" t="inlineStr">
@@ -60477,7 +60477,7 @@
       </c>
       <c r="CF194" s="24" t="inlineStr">
         <is>
-          <t>1.0089</t>
+          <t>1.0077</t>
         </is>
       </c>
       <c r="CG194" s="24" t="n"/>
@@ -60505,7 +60505,7 @@
       <c r="CQ194" s="24" t="n"/>
       <c r="CR194" s="24" t="inlineStr">
         <is>
-          <t>0.585723</t>
+          <t>0.58581</t>
         </is>
       </c>
       <c r="CS194" s="24" t="inlineStr">
@@ -60517,12 +60517,12 @@
     <row r="195" ht="36" customHeight="1">
       <c r="A195" s="24" t="inlineStr">
         <is>
-          <t>74cff5906ad44224</t>
+          <t>5e79dc4004814e2f</t>
         </is>
       </c>
       <c r="B195" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C195" s="24" t="inlineStr">
@@ -60567,23 +60567,23 @@
         </is>
       </c>
       <c r="L195" s="26" t="n">
-        <v>-115</v>
+        <v>-125</v>
       </c>
       <c r="M195" s="27" t="n">
-        <v>1.869565</v>
+        <v>1.8</v>
       </c>
       <c r="N195" s="28" t="n">
-        <v>0.534884</v>
+        <v>0.555556</v>
       </c>
       <c r="O195" s="28" t="n">
-        <v>0.5760999999999999</v>
+        <v>0.576188</v>
       </c>
       <c r="P195" s="28" t="n"/>
       <c r="Q195" s="28" t="n">
-        <v>0.041216</v>
+        <v>0.020632</v>
       </c>
       <c r="R195" s="26" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="S195" s="29" t="n">
         <v>0</v>
@@ -60609,7 +60609,7 @@
       <c r="AD195" s="24" t="n"/>
       <c r="AE195" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5350 (aec-mlb-cws-bos-2026-08-05); model edge vs ask +0.0411.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5550 (aec-mlb-cws-bos-2026-08-05); model edge vs ask +0.0212.</t>
         </is>
       </c>
       <c r="AF195" s="31" t="inlineStr">
@@ -60713,7 +60713,7 @@
       </c>
       <c r="BE195" s="24" t="inlineStr">
         <is>
-          <t>b747944f91650fd4</t>
+          <t>10f5b05f22dccd69</t>
         </is>
       </c>
       <c r="BF195" s="24" t="inlineStr">
@@ -60728,7 +60728,7 @@
       </c>
       <c r="BH195" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:57.825385Z</t>
+          <t>2026-08-05T13:52:29.150568Z</t>
         </is>
       </c>
       <c r="BI195" s="24" t="inlineStr">
@@ -60738,16 +60738,16 @@
       </c>
       <c r="BJ195" s="25" t="n"/>
       <c r="BK195" s="26" t="n">
-        <v>-115</v>
+        <v>-125</v>
       </c>
       <c r="BL195" s="27" t="n">
-        <v>1.869565</v>
+        <v>1.8</v>
       </c>
       <c r="BM195" s="28" t="n">
-        <v>0.534884</v>
+        <v>0.555556</v>
       </c>
       <c r="BN195" s="28" t="n">
-        <v>0.532338</v>
+        <v>0.552239</v>
       </c>
       <c r="BO195" s="28" t="n"/>
       <c r="BP195" s="25" t="n"/>
@@ -60780,7 +60780,7 @@
       </c>
       <c r="CF195" s="24" t="inlineStr">
         <is>
-          <t>1.0141</t>
+          <t>1.0129</t>
         </is>
       </c>
       <c r="CG195" s="24" t="n"/>
@@ -60808,7 +60808,7 @@
       <c r="CQ195" s="24" t="n"/>
       <c r="CR195" s="24" t="inlineStr">
         <is>
-          <t>0.5761</t>
+          <t>0.576188</t>
         </is>
       </c>
       <c r="CS195" s="24" t="inlineStr">
@@ -60820,12 +60820,12 @@
     <row r="196" ht="36" customHeight="1">
       <c r="A196" s="24" t="inlineStr">
         <is>
-          <t>e54060cb42344aa5</t>
+          <t>d1e30ef4ff0b4aa1</t>
         </is>
       </c>
       <c r="B196" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C196" s="24" t="inlineStr">
@@ -60879,11 +60879,11 @@
         <v>0.545455</v>
       </c>
       <c r="O196" s="28" t="n">
-        <v>0.59089</v>
+        <v>0.590933</v>
       </c>
       <c r="P196" s="28" t="n"/>
       <c r="Q196" s="28" t="n">
-        <v>0.045435</v>
+        <v>0.045478</v>
       </c>
       <c r="R196" s="26" t="n">
         <v>44</v>
@@ -61016,7 +61016,7 @@
       </c>
       <c r="BE196" s="24" t="inlineStr">
         <is>
-          <t>bb6f41cb5975b5bb</t>
+          <t>06a32b1aa50e018d</t>
         </is>
       </c>
       <c r="BF196" s="24" t="inlineStr">
@@ -61031,7 +61031,7 @@
       </c>
       <c r="BH196" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:58.789026Z</t>
+          <t>2026-08-05T13:52:29.624655Z</t>
         </is>
       </c>
       <c r="BI196" s="24" t="inlineStr">
@@ -61083,7 +61083,7 @@
       </c>
       <c r="CF196" s="24" t="inlineStr">
         <is>
-          <t>1.0072</t>
+          <t>1.0066</t>
         </is>
       </c>
       <c r="CG196" s="24" t="n"/>
@@ -61115,7 +61115,7 @@
       <c r="CQ196" s="24" t="n"/>
       <c r="CR196" s="24" t="inlineStr">
         <is>
-          <t>0.59089</t>
+          <t>0.590933</t>
         </is>
       </c>
       <c r="CS196" s="24" t="inlineStr">
@@ -61127,12 +61127,12 @@
     <row r="197" ht="36" customHeight="1">
       <c r="A197" s="24" t="inlineStr">
         <is>
-          <t>1f14ba2d3f6a4999</t>
+          <t>33f2e3a8a1e74278</t>
         </is>
       </c>
       <c r="B197" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C197" s="24" t="inlineStr">
@@ -61177,23 +61177,23 @@
         </is>
       </c>
       <c r="L197" s="26" t="n">
-        <v>-122</v>
+        <v>-125</v>
       </c>
       <c r="M197" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.8</v>
       </c>
       <c r="N197" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.555556</v>
       </c>
       <c r="O197" s="28" t="n">
         <v>0.6155080000000001</v>
       </c>
       <c r="P197" s="28" t="n"/>
       <c r="Q197" s="28" t="n">
-        <v>0.065958</v>
+        <v>0.059952</v>
       </c>
       <c r="R197" s="26" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="S197" s="29" t="n">
         <v>1.5</v>
@@ -61219,7 +61219,7 @@
       <c r="AD197" s="24" t="n"/>
       <c r="AE197" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5500 (aec-mlb-pit-mil-2026-08-05); model edge vs ask +0.0655.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5550 (aec-mlb-pit-mil-2026-08-05); model edge vs ask +0.0605.</t>
         </is>
       </c>
       <c r="AF197" s="31" t="inlineStr">
@@ -61338,7 +61338,7 @@
       </c>
       <c r="BH197" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:33:59.358107Z</t>
+          <t>2026-08-05T13:52:30.079092Z</t>
         </is>
       </c>
       <c r="BI197" s="24" t="inlineStr">
@@ -61348,16 +61348,16 @@
       </c>
       <c r="BJ197" s="25" t="n"/>
       <c r="BK197" s="26" t="n">
-        <v>-122</v>
+        <v>-125</v>
       </c>
       <c r="BL197" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.8</v>
       </c>
       <c r="BM197" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.555556</v>
       </c>
       <c r="BN197" s="28" t="n">
-        <v>0.547264</v>
+        <v>0.552239</v>
       </c>
       <c r="BO197" s="28" t="n"/>
       <c r="BP197" s="25" t="n"/>
@@ -61430,12 +61430,12 @@
     <row r="198" ht="36" customHeight="1">
       <c r="A198" s="24" t="inlineStr">
         <is>
-          <t>ac481a548c2d4c55</t>
+          <t>d43a3520d7d3492b</t>
         </is>
       </c>
       <c r="B198" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C198" s="24" t="inlineStr">
@@ -61480,23 +61480,23 @@
         </is>
       </c>
       <c r="L198" s="26" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="M198" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.884956</v>
       </c>
       <c r="N198" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.530516</v>
       </c>
       <c r="O198" s="28" t="n">
-        <v>0.5251209999999999</v>
+        <v>0.524802</v>
       </c>
       <c r="P198" s="28" t="n"/>
       <c r="Q198" s="28" t="n">
-        <v>0.00589</v>
+        <v>-0.005714</v>
       </c>
       <c r="R198" s="26" t="n">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="S198" s="29" t="n">
         <v>0</v>
@@ -61522,7 +61522,7 @@
       <c r="AD198" s="24" t="n"/>
       <c r="AE198" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5200 (aec-mlb-min-kc-2026-08-05); model edge vs ask +0.0051.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5300 (aec-mlb-min-kc-2026-08-05); model edge vs ask -0.0052.</t>
         </is>
       </c>
       <c r="AF198" s="31" t="inlineStr">
@@ -61626,7 +61626,7 @@
       </c>
       <c r="BE198" s="24" t="inlineStr">
         <is>
-          <t>f8ae77f69b137e22</t>
+          <t>420793a043fef772</t>
         </is>
       </c>
       <c r="BF198" s="24" t="inlineStr">
@@ -61641,7 +61641,7 @@
       </c>
       <c r="BH198" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:34:00.271972Z</t>
+          <t>2026-08-05T13:52:30.727273Z</t>
         </is>
       </c>
       <c r="BI198" s="24" t="inlineStr">
@@ -61651,16 +61651,16 @@
       </c>
       <c r="BJ198" s="25" t="n"/>
       <c r="BK198" s="26" t="n">
-        <v>-108</v>
+        <v>-113</v>
       </c>
       <c r="BL198" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.884956</v>
       </c>
       <c r="BM198" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.530516</v>
       </c>
       <c r="BN198" s="28" t="n">
-        <v>0.5148509999999999</v>
+        <v>0.527363</v>
       </c>
       <c r="BO198" s="28" t="n"/>
       <c r="BP198" s="25" t="n"/>
@@ -61693,7 +61693,7 @@
       </c>
       <c r="CF198" s="24" t="inlineStr">
         <is>
-          <t>1.0128</t>
+          <t>1.0171</t>
         </is>
       </c>
       <c r="CG198" s="24" t="n"/>
@@ -61721,24 +61721,24 @@
       <c r="CQ198" s="24" t="n"/>
       <c r="CR198" s="24" t="inlineStr">
         <is>
-          <t>0.525121</t>
+          <t>0.524802</t>
         </is>
       </c>
       <c r="CS198" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="199" ht="36" customHeight="1">
       <c r="A199" s="24" t="inlineStr">
         <is>
-          <t>360f9b23ece34b85</t>
+          <t>50fddafac55b4f3c</t>
         </is>
       </c>
       <c r="B199" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C199" s="24" t="inlineStr">
@@ -61783,23 +61783,23 @@
         </is>
       </c>
       <c r="L199" s="26" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="M199" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.694444</v>
       </c>
       <c r="N199" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.590164</v>
       </c>
       <c r="O199" s="28" t="n">
         <v>0.550053</v>
       </c>
       <c r="P199" s="28" t="n"/>
       <c r="Q199" s="28" t="n">
-        <v>-0.029779</v>
+        <v>-0.040111</v>
       </c>
       <c r="R199" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="S199" s="29" t="n">
         <v>0</v>
@@ -61825,7 +61825,7 @@
       <c r="AD199" s="24" t="n"/>
       <c r="AE199" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5800 (aec-mlb-det-sea-2026-08-05); model edge vs ask -0.0299.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5900 (aec-mlb-det-sea-2026-08-05); model edge vs ask -0.0399.</t>
         </is>
       </c>
       <c r="AF199" s="31" t="inlineStr">
@@ -61944,7 +61944,7 @@
       </c>
       <c r="BH199" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:34:01.074140Z</t>
+          <t>2026-08-05T13:52:31.897237Z</t>
         </is>
       </c>
       <c r="BI199" s="24" t="inlineStr">
@@ -61954,16 +61954,16 @@
       </c>
       <c r="BJ199" s="25" t="n"/>
       <c r="BK199" s="26" t="n">
-        <v>-138</v>
+        <v>-144</v>
       </c>
       <c r="BL199" s="27" t="n">
-        <v>1.724638</v>
+        <v>1.694444</v>
       </c>
       <c r="BM199" s="28" t="n">
-        <v>0.579832</v>
+        <v>0.590164</v>
       </c>
       <c r="BN199" s="28" t="n">
-        <v>0.577114</v>
+        <v>0.5870649999999999</v>
       </c>
       <c r="BO199" s="28" t="n"/>
       <c r="BP199" s="25" t="n"/>
@@ -62036,12 +62036,12 @@
     <row r="200" ht="36" customHeight="1">
       <c r="A200" s="24" t="inlineStr">
         <is>
-          <t>b5bac8a287c347f5</t>
+          <t>4304c4a91d1145b1</t>
         </is>
       </c>
       <c r="B200" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:35:50.664769Z</t>
+          <t>2026-08-05T13:54:09.180176Z</t>
         </is>
       </c>
       <c r="C200" s="24" t="inlineStr">
@@ -62086,23 +62086,23 @@
         </is>
       </c>
       <c r="L200" s="26" t="n">
-        <v>-111</v>
+        <v>-115</v>
       </c>
       <c r="M200" s="27" t="n">
-        <v>1.900901</v>
+        <v>1.869565</v>
       </c>
       <c r="N200" s="28" t="n">
-        <v>0.526066</v>
+        <v>0.534884</v>
       </c>
       <c r="O200" s="28" t="n">
         <v>0.512293</v>
       </c>
       <c r="P200" s="28" t="n"/>
       <c r="Q200" s="28" t="n">
-        <v>-0.013773</v>
+        <v>-0.022591</v>
       </c>
       <c r="R200" s="26" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="S200" s="29" t="n">
         <v>0</v>
@@ -62128,7 +62128,7 @@
       <c r="AD200" s="24" t="n"/>
       <c r="AE200" s="31" t="inlineStr">
         <is>
-          <t>Learned LR call at threshold 0.5873; executable ask 0.5250 (aec-mlb-sd-az-2026-08-05); model edge vs ask -0.0127.</t>
+          <t>Learned LR call at threshold 0.5873; executable ask 0.5350 (aec-mlb-sd-az-2026-08-05); model edge vs ask -0.0227.</t>
         </is>
       </c>
       <c r="AF200" s="31" t="inlineStr">
@@ -62247,7 +62247,7 @@
       </c>
       <c r="BH200" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:34:01.895512Z</t>
+          <t>2026-08-05T13:52:33.047392Z</t>
         </is>
       </c>
       <c r="BI200" s="24" t="inlineStr">
@@ -62257,16 +62257,16 @@
       </c>
       <c r="BJ200" s="25" t="n"/>
       <c r="BK200" s="26" t="n">
-        <v>-111</v>
+        <v>-115</v>
       </c>
       <c r="BL200" s="27" t="n">
-        <v>1.900901</v>
+        <v>1.869565</v>
       </c>
       <c r="BM200" s="28" t="n">
-        <v>0.526066</v>
+        <v>0.534884</v>
       </c>
       <c r="BN200" s="28" t="n">
-        <v>0.522388</v>
+        <v>0.532338</v>
       </c>
       <c r="BO200" s="28" t="n"/>
       <c r="BP200" s="25" t="n"/>
@@ -62339,12 +62339,12 @@
     <row r="201" ht="36" customHeight="1">
       <c r="A201" s="24" t="inlineStr">
         <is>
-          <t>2af2f4dcab2b4c21</t>
+          <t>b7732472266842a3</t>
         </is>
       </c>
       <c r="B201" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C201" s="24" t="inlineStr">
@@ -62391,25 +62391,25 @@
         </is>
       </c>
       <c r="L201" s="26" t="n">
-        <v>-135</v>
+        <v>-122</v>
       </c>
       <c r="M201" s="27" t="n">
-        <v>1.740741</v>
+        <v>1.819672</v>
       </c>
       <c r="N201" s="28" t="n">
-        <v>0.574468</v>
+        <v>0.54955</v>
       </c>
       <c r="O201" s="28" t="n">
-        <v>0.556045</v>
+        <v>0.554069</v>
       </c>
       <c r="P201" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q201" s="28" t="n">
-        <v>-0.018423</v>
+        <v>0.004519</v>
       </c>
       <c r="R201" s="26" t="n">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="S201" s="29" t="n">
         <v>1</v>
@@ -62435,7 +62435,7 @@
       <c r="AD201" s="24" t="n"/>
       <c r="AE201" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.45-5.29; raw selected-side p=0.5823, calibrated p=0.5560.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.45-5.29; raw selected-side p=0.5794, calibrated p=0.5541.</t>
         </is>
       </c>
       <c r="AF201" s="31" t="inlineStr">
@@ -62554,7 +62554,7 @@
       </c>
       <c r="BH201" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI201" s="24" t="inlineStr">
@@ -62566,16 +62566,16 @@
         <v>1.5</v>
       </c>
       <c r="BK201" s="26" t="n">
-        <v>-135</v>
+        <v>-122</v>
       </c>
       <c r="BL201" s="27" t="n">
-        <v>1.740741</v>
+        <v>1.819672</v>
       </c>
       <c r="BM201" s="28" t="n">
-        <v>0.574468</v>
+        <v>0.54955</v>
       </c>
       <c r="BN201" s="28" t="n">
-        <v>0.572139</v>
+        <v>0.547264</v>
       </c>
       <c r="BO201" s="28" t="n"/>
       <c r="BP201" s="25" t="n"/>
@@ -62609,19 +62609,19 @@
       <c r="CR201" s="24" t="n"/>
       <c r="CS201" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="202" ht="36" customHeight="1">
       <c r="A202" s="24" t="inlineStr">
         <is>
-          <t>2e28c6f185954677</t>
+          <t>d6db2f4b521b400d</t>
         </is>
       </c>
       <c r="B202" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C202" s="24" t="inlineStr">
@@ -62677,13 +62677,13 @@
         <v>0.473934</v>
       </c>
       <c r="O202" s="28" t="n">
-        <v>0.524815</v>
+        <v>0.525275</v>
       </c>
       <c r="P202" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q202" s="28" t="n">
-        <v>0.050881</v>
+        <v>0.051341</v>
       </c>
       <c r="R202" s="26" t="n">
         <v>51</v>
@@ -62712,7 +62712,7 @@
       <c r="AD202" s="24" t="n"/>
       <c r="AE202" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.45-5.29; raw selected-side p=0.5766, calibrated p=0.5248.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.45-5.29; raw selected-side p=0.5784, calibrated p=0.5253.</t>
         </is>
       </c>
       <c r="AF202" s="31" t="inlineStr">
@@ -62831,7 +62831,7 @@
       </c>
       <c r="BH202" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI202" s="24" t="inlineStr">
@@ -62893,12 +62893,12 @@
     <row r="203" ht="36" customHeight="1">
       <c r="A203" s="24" t="inlineStr">
         <is>
-          <t>f2a4bd8da10e45d5</t>
+          <t>433e220b206847ba</t>
         </is>
       </c>
       <c r="B203" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C203" s="24" t="inlineStr">
@@ -62933,7 +62933,7 @@
       </c>
       <c r="I203" s="24" t="inlineStr">
         <is>
-          <t>home</t>
+          <t>away</t>
         </is>
       </c>
       <c r="J203" s="25" t="n">
@@ -62954,19 +62954,19 @@
         <v>0.635036</v>
       </c>
       <c r="O203" s="28" t="n">
-        <v>0.6607420000000001</v>
+        <v>0.576862</v>
       </c>
       <c r="P203" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q203" s="28" t="n">
-        <v>0.025706</v>
+        <v>-0.058174</v>
       </c>
       <c r="R203" s="26" t="n">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="S203" s="29" t="n">
-        <v>1.75</v>
+        <v>1.25</v>
       </c>
       <c r="T203" s="24" t="inlineStr">
         <is>
@@ -62989,7 +62989,7 @@
       <c r="AD203" s="24" t="n"/>
       <c r="AE203" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 3.96-4.59; raw selected-side p=0.7359, calibrated p=0.6607.</t>
+          <t>Measured Edge Margin: Trend Engine projected 3.96-4.59; raw selected-side p=0.6128, calibrated p=0.5769.</t>
         </is>
       </c>
       <c r="AF203" s="31" t="inlineStr">
@@ -63108,7 +63108,7 @@
       </c>
       <c r="BH203" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI203" s="24" t="inlineStr">
@@ -63163,19 +63163,19 @@
       <c r="CR203" s="24" t="n"/>
       <c r="CS203" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="204" ht="36" customHeight="1">
       <c r="A204" s="24" t="inlineStr">
         <is>
-          <t>3bc0a1dfe50a4d9e</t>
+          <t>10263ec937d04c88</t>
         </is>
       </c>
       <c r="B204" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C204" s="24" t="inlineStr">
@@ -63222,25 +63222,25 @@
         </is>
       </c>
       <c r="L204" s="26" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="M204" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.961538</v>
       </c>
       <c r="N204" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.509804</v>
       </c>
       <c r="O204" s="28" t="n">
-        <v>0.539558</v>
+        <v>0.540166</v>
       </c>
       <c r="P204" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q204" s="28" t="n">
-        <v>0.020327</v>
+        <v>0.030362</v>
       </c>
       <c r="R204" s="26" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="S204" s="29" t="n">
         <v>1</v>
@@ -63266,7 +63266,7 @@
       <c r="AD204" s="24" t="n"/>
       <c r="AE204" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 3.96-4.59; raw selected-side p=0.6359, calibrated p=0.5396.</t>
+          <t>Measured Edge Totals: Trend Engine projected 3.96-4.59; raw selected-side p=0.6383, calibrated p=0.5402.</t>
         </is>
       </c>
       <c r="AF204" s="31" t="inlineStr">
@@ -63385,7 +63385,7 @@
       </c>
       <c r="BH204" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI204" s="24" t="inlineStr">
@@ -63397,16 +63397,16 @@
         <v>9.5</v>
       </c>
       <c r="BK204" s="26" t="n">
-        <v>-108</v>
+        <v>-104</v>
       </c>
       <c r="BL204" s="27" t="n">
-        <v>1.925926</v>
+        <v>1.961538</v>
       </c>
       <c r="BM204" s="28" t="n">
-        <v>0.519231</v>
+        <v>0.509804</v>
       </c>
       <c r="BN204" s="28" t="n">
-        <v>0.517413</v>
+        <v>0.507463</v>
       </c>
       <c r="BO204" s="28" t="n"/>
       <c r="BP204" s="25" t="n"/>
@@ -63447,12 +63447,12 @@
     <row r="205" ht="36" customHeight="1">
       <c r="A205" s="24" t="inlineStr">
         <is>
-          <t>0d24c94754b64c63</t>
+          <t>21ae370f36684ead</t>
         </is>
       </c>
       <c r="B205" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C205" s="24" t="inlineStr">
@@ -63508,13 +63508,13 @@
         <v>0.565217</v>
       </c>
       <c r="O205" s="28" t="n">
-        <v>0.588514</v>
+        <v>0.587935</v>
       </c>
       <c r="P205" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q205" s="28" t="n">
-        <v>0.023297</v>
+        <v>0.022718</v>
       </c>
       <c r="R205" s="26" t="n">
         <v>32</v>
@@ -63543,7 +63543,7 @@
       <c r="AD205" s="24" t="n"/>
       <c r="AE205" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.57-4.92; raw selected-side p=0.6299, calibrated p=0.5885.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.57-4.92; raw selected-side p=0.6290, calibrated p=0.5879.</t>
         </is>
       </c>
       <c r="AF205" s="31" t="inlineStr">
@@ -63662,7 +63662,7 @@
       </c>
       <c r="BH205" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI205" s="24" t="inlineStr">
@@ -63724,12 +63724,12 @@
     <row r="206" ht="36" customHeight="1">
       <c r="A206" s="24" t="inlineStr">
         <is>
-          <t>76748dfba8094a58</t>
+          <t>5ddca6a6a2a64ce9</t>
         </is>
       </c>
       <c r="B206" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C206" s="24" t="inlineStr">
@@ -63785,16 +63785,16 @@
         <v>0.480769</v>
       </c>
       <c r="O206" s="28" t="n">
-        <v>0.522257</v>
+        <v>0.519176</v>
       </c>
       <c r="P206" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q206" s="28" t="n">
-        <v>0.041488</v>
+        <v>0.038407</v>
       </c>
       <c r="R206" s="26" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="S206" s="29" t="n">
         <v>1</v>
@@ -63820,7 +63820,7 @@
       <c r="AD206" s="24" t="n"/>
       <c r="AE206" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.57-4.92; raw selected-side p=0.5663, calibrated p=0.5223.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.57-4.92; raw selected-side p=0.5538, calibrated p=0.5192.</t>
         </is>
       </c>
       <c r="AF206" s="31" t="inlineStr">
@@ -63939,7 +63939,7 @@
       </c>
       <c r="BH206" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI206" s="24" t="inlineStr">
@@ -64001,12 +64001,12 @@
     <row r="207" ht="36" customHeight="1">
       <c r="A207" s="24" t="inlineStr">
         <is>
-          <t>0cd90ea61a734a0b</t>
+          <t>011175b8945c4b41</t>
         </is>
       </c>
       <c r="B207" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C207" s="24" t="inlineStr">
@@ -64053,25 +64053,25 @@
         </is>
       </c>
       <c r="L207" s="26" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="M207" s="27" t="n">
-        <v>1.961538</v>
+        <v>2</v>
       </c>
       <c r="N207" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.5</v>
       </c>
       <c r="O207" s="28" t="n">
-        <v>0.602278</v>
+        <v>0.600915</v>
       </c>
       <c r="P207" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q207" s="28" t="n">
-        <v>0.092474</v>
+        <v>0.100915</v>
       </c>
       <c r="R207" s="26" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="S207" s="29" t="n">
         <v>1.5</v>
@@ -64097,7 +64097,7 @@
       <c r="AD207" s="24" t="n"/>
       <c r="AE207" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.81-4.67; raw selected-side p=0.6501, calibrated p=0.6023.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.81-4.66; raw selected-side p=0.6481, calibrated p=0.6009.</t>
         </is>
       </c>
       <c r="AF207" s="31" t="inlineStr">
@@ -64216,7 +64216,7 @@
       </c>
       <c r="BH207" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI207" s="24" t="inlineStr">
@@ -64228,16 +64228,16 @@
         <v>1.5</v>
       </c>
       <c r="BK207" s="26" t="n">
-        <v>-104</v>
+        <v>100</v>
       </c>
       <c r="BL207" s="27" t="n">
-        <v>1.961538</v>
+        <v>2</v>
       </c>
       <c r="BM207" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.5</v>
       </c>
       <c r="BN207" s="28" t="n">
-        <v>0.507463</v>
+        <v>0.497512</v>
       </c>
       <c r="BO207" s="28" t="n"/>
       <c r="BP207" s="25" t="n"/>
@@ -64278,12 +64278,12 @@
     <row r="208" ht="36" customHeight="1">
       <c r="A208" s="24" t="inlineStr">
         <is>
-          <t>14659c36acee4d5f</t>
+          <t>b0eee51cd3b44422</t>
         </is>
       </c>
       <c r="B208" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C208" s="24" t="inlineStr">
@@ -64330,25 +64330,25 @@
         </is>
       </c>
       <c r="L208" s="26" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M208" s="27" t="n">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="N208" s="28" t="n">
-        <v>0.5</v>
+        <v>0.49505</v>
       </c>
       <c r="O208" s="28" t="n">
-        <v>0.557989</v>
+        <v>0.558548</v>
       </c>
       <c r="P208" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q208" s="28" t="n">
-        <v>0.057989</v>
+        <v>0.063498</v>
       </c>
       <c r="R208" s="26" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="S208" s="29" t="n">
         <v>1</v>
@@ -64374,7 +64374,7 @@
       <c r="AD208" s="24" t="n"/>
       <c r="AE208" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.81-4.67; raw selected-side p=0.7101, calibrated p=0.5580.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.81-4.66; raw selected-side p=0.7124, calibrated p=0.5585.</t>
         </is>
       </c>
       <c r="AF208" s="31" t="inlineStr">
@@ -64493,7 +64493,7 @@
       </c>
       <c r="BH208" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI208" s="24" t="inlineStr">
@@ -64505,16 +64505,16 @@
         <v>11.5</v>
       </c>
       <c r="BK208" s="26" t="n">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="BL208" s="27" t="n">
-        <v>2</v>
+        <v>2.02</v>
       </c>
       <c r="BM208" s="28" t="n">
-        <v>0.5</v>
+        <v>0.49505</v>
       </c>
       <c r="BN208" s="28" t="n">
-        <v>0.49505</v>
+        <v>0.492537</v>
       </c>
       <c r="BO208" s="28" t="n"/>
       <c r="BP208" s="25" t="n"/>
@@ -64555,12 +64555,12 @@
     <row r="209" ht="36" customHeight="1">
       <c r="A209" s="24" t="inlineStr">
         <is>
-          <t>c84c5e3ee91443f5</t>
+          <t>087961e2f0c74b71</t>
         </is>
       </c>
       <c r="B209" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C209" s="24" t="inlineStr">
@@ -64607,25 +64607,25 @@
         </is>
       </c>
       <c r="L209" s="26" t="n">
-        <v>-167</v>
+        <v>-174</v>
       </c>
       <c r="M209" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.574713</v>
       </c>
       <c r="N209" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.635036</v>
       </c>
       <c r="O209" s="28" t="n">
-        <v>0.585379</v>
+        <v>0.590183</v>
       </c>
       <c r="P209" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q209" s="28" t="n">
-        <v>-0.040089</v>
+        <v>-0.044853</v>
       </c>
       <c r="R209" s="26" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="S209" s="29" t="n">
         <v>1.25</v>
@@ -64651,7 +64651,7 @@
       <c r="AD209" s="24" t="n"/>
       <c r="AE209" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.25-4.70; raw selected-side p=0.6253, calibrated p=0.5854.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.25-4.70; raw selected-side p=0.6323, calibrated p=0.5902.</t>
         </is>
       </c>
       <c r="AF209" s="31" t="inlineStr">
@@ -64770,7 +64770,7 @@
       </c>
       <c r="BH209" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI209" s="24" t="inlineStr">
@@ -64782,16 +64782,16 @@
         <v>1.5</v>
       </c>
       <c r="BK209" s="26" t="n">
-        <v>-167</v>
+        <v>-174</v>
       </c>
       <c r="BL209" s="27" t="n">
-        <v>1.598802</v>
+        <v>1.574713</v>
       </c>
       <c r="BM209" s="28" t="n">
-        <v>0.625468</v>
+        <v>0.635036</v>
       </c>
       <c r="BN209" s="28" t="n">
-        <v>0.621891</v>
+        <v>0.631841</v>
       </c>
       <c r="BO209" s="28" t="n"/>
       <c r="BP209" s="25" t="n"/>
@@ -64832,12 +64832,12 @@
     <row r="210" ht="36" customHeight="1">
       <c r="A210" s="24" t="inlineStr">
         <is>
-          <t>276c399a45f44a14</t>
+          <t>535a08003a8a4c2d</t>
         </is>
       </c>
       <c r="B210" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C210" s="24" t="inlineStr">
@@ -64876,7 +64876,7 @@
         </is>
       </c>
       <c r="J210" s="25" t="n">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="K210" s="24" t="inlineStr">
         <is>
@@ -64884,25 +64884,25 @@
         </is>
       </c>
       <c r="L210" s="26" t="n">
-        <v>111</v>
+        <v>-115</v>
       </c>
       <c r="M210" s="27" t="n">
-        <v>2.11</v>
+        <v>1.869565</v>
       </c>
       <c r="N210" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.534884</v>
       </c>
       <c r="O210" s="28" t="n">
-        <v>0.5089669999999999</v>
+        <v>0.527597</v>
       </c>
       <c r="P210" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q210" s="28" t="n">
-        <v>0.035033</v>
+        <v>-0.007287</v>
       </c>
       <c r="R210" s="26" t="n">
-        <v>43</v>
+        <v>22</v>
       </c>
       <c r="S210" s="29" t="n">
         <v>1</v>
@@ -64928,7 +64928,7 @@
       <c r="AD210" s="24" t="n"/>
       <c r="AE210" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.25-4.70; raw selected-side p=0.5128, calibrated p=0.5090.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.25-4.70; raw selected-side p=0.5877, calibrated p=0.5276.</t>
         </is>
       </c>
       <c r="AF210" s="31" t="inlineStr">
@@ -65047,7 +65047,7 @@
       </c>
       <c r="BH210" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI210" s="24" t="inlineStr">
@@ -65056,19 +65056,19 @@
         </is>
       </c>
       <c r="BJ210" s="25" t="n">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="BK210" s="26" t="n">
-        <v>111</v>
+        <v>-115</v>
       </c>
       <c r="BL210" s="27" t="n">
-        <v>2.11</v>
+        <v>1.869565</v>
       </c>
       <c r="BM210" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.534884</v>
       </c>
       <c r="BN210" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.532338</v>
       </c>
       <c r="BO210" s="28" t="n"/>
       <c r="BP210" s="25" t="n"/>
@@ -65102,19 +65102,19 @@
       <c r="CR210" s="24" t="n"/>
       <c r="CS210" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="211" ht="36" customHeight="1">
       <c r="A211" s="24" t="inlineStr">
         <is>
-          <t>09e9149787ed47e4</t>
+          <t>ed818bf10f91467f</t>
         </is>
       </c>
       <c r="B211" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C211" s="24" t="inlineStr">
@@ -65170,16 +65170,16 @@
         <v>0.604743</v>
       </c>
       <c r="O211" s="28" t="n">
-        <v>0.590797</v>
+        <v>0.594067</v>
       </c>
       <c r="P211" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q211" s="28" t="n">
-        <v>-0.013946</v>
+        <v>-0.010676</v>
       </c>
       <c r="R211" s="26" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S211" s="29" t="n">
         <v>1.25</v>
@@ -65205,7 +65205,7 @@
       <c r="AD211" s="24" t="n"/>
       <c r="AE211" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.90-5.09; raw selected-side p=0.6332, calibrated p=0.5908.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.90-5.09; raw selected-side p=0.6381, calibrated p=0.5941.</t>
         </is>
       </c>
       <c r="AF211" s="31" t="inlineStr">
@@ -65324,7 +65324,7 @@
       </c>
       <c r="BH211" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI211" s="24" t="inlineStr">
@@ -65386,12 +65386,12 @@
     <row r="212" ht="36" customHeight="1">
       <c r="A212" s="24" t="inlineStr">
         <is>
-          <t>c5aaf24102e945be</t>
+          <t>b1ad3a4710984315</t>
         </is>
       </c>
       <c r="B212" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C212" s="24" t="inlineStr">
@@ -65447,16 +65447,16 @@
         <v>0.490196</v>
       </c>
       <c r="O212" s="28" t="n">
-        <v>0.509116</v>
+        <v>0.509961</v>
       </c>
       <c r="P212" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q212" s="28" t="n">
-        <v>0.01892</v>
+        <v>0.019765</v>
       </c>
       <c r="R212" s="26" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="S212" s="29" t="n">
         <v>1</v>
@@ -65482,7 +65482,7 @@
       <c r="AD212" s="24" t="n"/>
       <c r="AE212" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.90-5.09; raw selected-side p=0.5133, calibrated p=0.5091.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.90-5.09; raw selected-side p=0.5168, calibrated p=0.5100.</t>
         </is>
       </c>
       <c r="AF212" s="31" t="inlineStr">
@@ -65601,7 +65601,7 @@
       </c>
       <c r="BH212" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI212" s="24" t="inlineStr">
@@ -65663,12 +65663,12 @@
     <row r="213" ht="36" customHeight="1">
       <c r="A213" s="24" t="inlineStr">
         <is>
-          <t>066b2518b950478a</t>
+          <t>09d22d46c62d4d23</t>
         </is>
       </c>
       <c r="B213" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C213" s="24" t="inlineStr">
@@ -65715,25 +65715,25 @@
         </is>
       </c>
       <c r="L213" s="26" t="n">
-        <v>-153</v>
+        <v>-170</v>
       </c>
       <c r="M213" s="27" t="n">
-        <v>1.653595</v>
+        <v>1.588235</v>
       </c>
       <c r="N213" s="28" t="n">
-        <v>0.604743</v>
+        <v>0.62963</v>
       </c>
       <c r="O213" s="28" t="n">
-        <v>0.60221</v>
+        <v>0.611375</v>
       </c>
       <c r="P213" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q213" s="28" t="n">
-        <v>-0.002533</v>
+        <v>-0.018255</v>
       </c>
       <c r="R213" s="26" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="S213" s="29" t="n">
         <v>1.5</v>
@@ -65759,7 +65759,7 @@
       <c r="AD213" s="24" t="n"/>
       <c r="AE213" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.46-4.24; raw selected-side p=0.6500, calibrated p=0.6022.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.46-4.24; raw selected-side p=0.6634, calibrated p=0.6114.</t>
         </is>
       </c>
       <c r="AF213" s="31" t="inlineStr">
@@ -65878,7 +65878,7 @@
       </c>
       <c r="BH213" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI213" s="24" t="inlineStr">
@@ -65890,16 +65890,16 @@
         <v>1.5</v>
       </c>
       <c r="BK213" s="26" t="n">
-        <v>-153</v>
+        <v>-170</v>
       </c>
       <c r="BL213" s="27" t="n">
-        <v>1.653595</v>
+        <v>1.588235</v>
       </c>
       <c r="BM213" s="28" t="n">
-        <v>0.604743</v>
+        <v>0.62963</v>
       </c>
       <c r="BN213" s="28" t="n">
-        <v>0.60199</v>
+        <v>0.626866</v>
       </c>
       <c r="BO213" s="28" t="n"/>
       <c r="BP213" s="25" t="n"/>
@@ -65940,12 +65940,12 @@
     <row r="214" ht="36" customHeight="1">
       <c r="A214" s="24" t="inlineStr">
         <is>
-          <t>c8fc1ee12e1f422d</t>
+          <t>e753f321748a4b0a</t>
         </is>
       </c>
       <c r="B214" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C214" s="24" t="inlineStr">
@@ -65980,11 +65980,11 @@
       </c>
       <c r="I214" s="24" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>over</t>
         </is>
       </c>
       <c r="J214" s="25" t="n">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="K214" s="24" t="inlineStr">
         <is>
@@ -65992,25 +65992,25 @@
         </is>
       </c>
       <c r="L214" s="26" t="n">
-        <v>-102</v>
+        <v>-111</v>
       </c>
       <c r="M214" s="27" t="n">
-        <v>1.980392</v>
+        <v>1.900901</v>
       </c>
       <c r="N214" s="28" t="n">
-        <v>0.50495</v>
+        <v>0.526066</v>
       </c>
       <c r="O214" s="28" t="n">
-        <v>0.50934</v>
+        <v>0.522244</v>
       </c>
       <c r="P214" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q214" s="28" t="n">
-        <v>0.00439</v>
+        <v>-0.003822</v>
       </c>
       <c r="R214" s="26" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="S214" s="29" t="n">
         <v>1</v>
@@ -66036,7 +66036,7 @@
       <c r="AD214" s="24" t="n"/>
       <c r="AE214" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.46-4.24; raw selected-side p=0.5142, calibrated p=0.5093.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.46-4.24; raw selected-side p=0.5662, calibrated p=0.5222.</t>
         </is>
       </c>
       <c r="AF214" s="31" t="inlineStr">
@@ -66155,7 +66155,7 @@
       </c>
       <c r="BH214" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI214" s="24" t="inlineStr">
@@ -66164,19 +66164,19 @@
         </is>
       </c>
       <c r="BJ214" s="25" t="n">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="BK214" s="26" t="n">
-        <v>-102</v>
+        <v>-111</v>
       </c>
       <c r="BL214" s="27" t="n">
-        <v>1.980392</v>
+        <v>1.900901</v>
       </c>
       <c r="BM214" s="28" t="n">
-        <v>0.50495</v>
+        <v>0.526066</v>
       </c>
       <c r="BN214" s="28" t="n">
-        <v>0.502488</v>
+        <v>0.522388</v>
       </c>
       <c r="BO214" s="28" t="n"/>
       <c r="BP214" s="25" t="n"/>
@@ -66210,19 +66210,19 @@
       <c r="CR214" s="24" t="n"/>
       <c r="CS214" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="215" ht="36" customHeight="1">
       <c r="A215" s="24" t="inlineStr">
         <is>
-          <t>752d0681afe84a29</t>
+          <t>3d42118f96554a28</t>
         </is>
       </c>
       <c r="B215" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C215" s="24" t="inlineStr">
@@ -66269,25 +66269,25 @@
         </is>
       </c>
       <c r="L215" s="26" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="M215" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.819672</v>
       </c>
       <c r="N215" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.54955</v>
       </c>
       <c r="O215" s="28" t="n">
-        <v>0.60238</v>
+        <v>0.603096</v>
       </c>
       <c r="P215" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q215" s="28" t="n">
-        <v>0.042909</v>
+        <v>0.053546</v>
       </c>
       <c r="R215" s="26" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="S215" s="29" t="n">
         <v>1.5</v>
@@ -66313,7 +66313,7 @@
       <c r="AD215" s="24" t="n"/>
       <c r="AE215" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 5.21-5.30; raw selected-side p=0.6502, calibrated p=0.6024.</t>
+          <t>Measured Edge Margin: Trend Engine projected 5.21-5.30; raw selected-side p=0.6513, calibrated p=0.6031.</t>
         </is>
       </c>
       <c r="AF215" s="31" t="inlineStr">
@@ -66432,7 +66432,7 @@
       </c>
       <c r="BH215" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI215" s="24" t="inlineStr">
@@ -66444,16 +66444,16 @@
         <v>1.5</v>
       </c>
       <c r="BK215" s="26" t="n">
-        <v>-127</v>
+        <v>-122</v>
       </c>
       <c r="BL215" s="27" t="n">
-        <v>1.787402</v>
+        <v>1.819672</v>
       </c>
       <c r="BM215" s="28" t="n">
-        <v>0.5594710000000001</v>
+        <v>0.54955</v>
       </c>
       <c r="BN215" s="28" t="n">
-        <v>0.554455</v>
+        <v>0.547264</v>
       </c>
       <c r="BO215" s="28" t="n"/>
       <c r="BP215" s="25" t="n"/>
@@ -66494,12 +66494,12 @@
     <row r="216" ht="36" customHeight="1">
       <c r="A216" s="24" t="inlineStr">
         <is>
-          <t>aef861b91af148b0</t>
+          <t>5bd846da30024e77</t>
         </is>
       </c>
       <c r="B216" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C216" s="24" t="inlineStr">
@@ -66546,22 +66546,22 @@
         </is>
       </c>
       <c r="L216" s="26" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="M216" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.980392</v>
       </c>
       <c r="N216" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.50495</v>
       </c>
       <c r="O216" s="28" t="n">
-        <v>0.5154879999999999</v>
+        <v>0.511737</v>
       </c>
       <c r="P216" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q216" s="28" t="n">
-        <v>0.005684</v>
+        <v>0.006787</v>
       </c>
       <c r="R216" s="26" t="n">
         <v>29</v>
@@ -66590,7 +66590,7 @@
       <c r="AD216" s="24" t="n"/>
       <c r="AE216" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 5.21-5.30; raw selected-side p=0.5390, calibrated p=0.5155.</t>
+          <t>Measured Edge Totals: Trend Engine projected 5.21-5.30; raw selected-side p=0.5239, calibrated p=0.5117.</t>
         </is>
       </c>
       <c r="AF216" s="31" t="inlineStr">
@@ -66709,7 +66709,7 @@
       </c>
       <c r="BH216" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI216" s="24" t="inlineStr">
@@ -66721,16 +66721,16 @@
         <v>9.5</v>
       </c>
       <c r="BK216" s="26" t="n">
-        <v>-104</v>
+        <v>-102</v>
       </c>
       <c r="BL216" s="27" t="n">
-        <v>1.961538</v>
+        <v>1.980392</v>
       </c>
       <c r="BM216" s="28" t="n">
-        <v>0.509804</v>
+        <v>0.50495</v>
       </c>
       <c r="BN216" s="28" t="n">
-        <v>0.507463</v>
+        <v>0.502488</v>
       </c>
       <c r="BO216" s="28" t="n"/>
       <c r="BP216" s="25" t="n"/>
@@ -66771,12 +66771,12 @@
     <row r="217" ht="36" customHeight="1">
       <c r="A217" s="24" t="inlineStr">
         <is>
-          <t>52aaeb284bef4334</t>
+          <t>a08d34f0b56a4205</t>
         </is>
       </c>
       <c r="B217" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C217" s="24" t="inlineStr">
@@ -66823,25 +66823,25 @@
         </is>
       </c>
       <c r="L217" s="26" t="n">
-        <v>-150</v>
+        <v>-144</v>
       </c>
       <c r="M217" s="27" t="n">
-        <v>1.666667</v>
+        <v>1.694444</v>
       </c>
       <c r="N217" s="28" t="n">
-        <v>0.6</v>
+        <v>0.590164</v>
       </c>
       <c r="O217" s="28" t="n">
-        <v>0.6248320000000001</v>
+        <v>0.624219</v>
       </c>
       <c r="P217" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q217" s="28" t="n">
-        <v>0.024832</v>
+        <v>0.034055</v>
       </c>
       <c r="R217" s="26" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="S217" s="29" t="n">
         <v>1.5</v>
@@ -66867,7 +66867,7 @@
       <c r="AD217" s="24" t="n"/>
       <c r="AE217" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.74-4.57; raw selected-side p=0.6832, calibrated p=0.6248.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.74-4.57; raw selected-side p=0.6823, calibrated p=0.6242.</t>
         </is>
       </c>
       <c r="AF217" s="31" t="inlineStr">
@@ -66986,7 +66986,7 @@
       </c>
       <c r="BH217" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI217" s="24" t="inlineStr">
@@ -66998,16 +66998,16 @@
         <v>1.5</v>
       </c>
       <c r="BK217" s="26" t="n">
-        <v>-150</v>
+        <v>-144</v>
       </c>
       <c r="BL217" s="27" t="n">
-        <v>1.666667</v>
+        <v>1.694444</v>
       </c>
       <c r="BM217" s="28" t="n">
-        <v>0.6</v>
+        <v>0.590164</v>
       </c>
       <c r="BN217" s="28" t="n">
-        <v>0.597015</v>
+        <v>0.5870649999999999</v>
       </c>
       <c r="BO217" s="28" t="n"/>
       <c r="BP217" s="25" t="n"/>
@@ -67048,12 +67048,12 @@
     <row r="218" ht="36" customHeight="1">
       <c r="A218" s="24" t="inlineStr">
         <is>
-          <t>f40f762a1ba74bba</t>
+          <t>44d845a6727d4325</t>
         </is>
       </c>
       <c r="B218" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C218" s="24" t="inlineStr">
@@ -67100,25 +67100,25 @@
         </is>
       </c>
       <c r="L218" s="26" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="M218" s="27" t="n">
-        <v>1.900901</v>
+        <v>1.925926</v>
       </c>
       <c r="N218" s="28" t="n">
-        <v>0.526066</v>
+        <v>0.519231</v>
       </c>
       <c r="O218" s="28" t="n">
-        <v>0.516866</v>
+        <v>0.515997</v>
       </c>
       <c r="P218" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q218" s="28" t="n">
-        <v>-0.0092</v>
+        <v>-0.003234</v>
       </c>
       <c r="R218" s="26" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="S218" s="29" t="n">
         <v>1</v>
@@ -67144,7 +67144,7 @@
       <c r="AD218" s="24" t="n"/>
       <c r="AE218" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.74-4.57; raw selected-side p=0.5445, calibrated p=0.5169.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.74-4.57; raw selected-side p=0.5411, calibrated p=0.5160.</t>
         </is>
       </c>
       <c r="AF218" s="31" t="inlineStr">
@@ -67263,7 +67263,7 @@
       </c>
       <c r="BH218" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI218" s="24" t="inlineStr">
@@ -67275,16 +67275,16 @@
         <v>8.5</v>
       </c>
       <c r="BK218" s="26" t="n">
-        <v>-111</v>
+        <v>-108</v>
       </c>
       <c r="BL218" s="27" t="n">
-        <v>1.900901</v>
+        <v>1.925926</v>
       </c>
       <c r="BM218" s="28" t="n">
-        <v>0.526066</v>
+        <v>0.519231</v>
       </c>
       <c r="BN218" s="28" t="n">
-        <v>0.522388</v>
+        <v>0.517413</v>
       </c>
       <c r="BO218" s="28" t="n"/>
       <c r="BP218" s="25" t="n"/>
@@ -67325,12 +67325,12 @@
     <row r="219" ht="36" customHeight="1">
       <c r="A219" s="24" t="inlineStr">
         <is>
-          <t>bb089dab22964210</t>
+          <t>05636342c84641d7</t>
         </is>
       </c>
       <c r="B219" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C219" s="24" t="inlineStr">
@@ -67377,25 +67377,25 @@
         </is>
       </c>
       <c r="L219" s="26" t="n">
-        <v>-182</v>
+        <v>-167</v>
       </c>
       <c r="M219" s="27" t="n">
-        <v>1.549451</v>
+        <v>1.598802</v>
       </c>
       <c r="N219" s="28" t="n">
-        <v>0.64539</v>
+        <v>0.625468</v>
       </c>
       <c r="O219" s="28" t="n">
-        <v>0.6332140000000001</v>
+        <v>0.633248</v>
       </c>
       <c r="P219" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q219" s="28" t="n">
-        <v>-0.012176</v>
+        <v>0.00778</v>
       </c>
       <c r="R219" s="26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="S219" s="29" t="n">
         <v>1.5</v>
@@ -67421,7 +67421,7 @@
       <c r="AD219" s="24" t="n"/>
       <c r="AE219" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.13-3.98; raw selected-side p=0.6955, calibrated p=0.6332.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.13-3.98; raw selected-side p=0.6956, calibrated p=0.6332.</t>
         </is>
       </c>
       <c r="AF219" s="31" t="inlineStr">
@@ -67540,7 +67540,7 @@
       </c>
       <c r="BH219" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI219" s="24" t="inlineStr">
@@ -67552,16 +67552,16 @@
         <v>1.5</v>
       </c>
       <c r="BK219" s="26" t="n">
-        <v>-182</v>
+        <v>-167</v>
       </c>
       <c r="BL219" s="27" t="n">
-        <v>1.549451</v>
+        <v>1.598802</v>
       </c>
       <c r="BM219" s="28" t="n">
-        <v>0.64539</v>
+        <v>0.625468</v>
       </c>
       <c r="BN219" s="28" t="n">
-        <v>0.641791</v>
+        <v>0.621891</v>
       </c>
       <c r="BO219" s="28" t="n"/>
       <c r="BP219" s="25" t="n"/>
@@ -67595,19 +67595,19 @@
       <c r="CR219" s="24" t="n"/>
       <c r="CS219" s="24" t="inlineStr">
         <is>
-          <t>False</t>
+          <t>True</t>
         </is>
       </c>
     </row>
     <row r="220" ht="36" customHeight="1">
       <c r="A220" s="24" t="inlineStr">
         <is>
-          <t>c4dda4d6947e4af2</t>
+          <t>0862f28e8fcd401c</t>
         </is>
       </c>
       <c r="B220" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C220" s="24" t="inlineStr">
@@ -67654,25 +67654,25 @@
         </is>
       </c>
       <c r="L220" s="26" t="n">
-        <v>100</v>
+        <v>-111</v>
       </c>
       <c r="M220" s="27" t="n">
-        <v>2</v>
+        <v>1.900901</v>
       </c>
       <c r="N220" s="28" t="n">
-        <v>0.5</v>
+        <v>0.526066</v>
       </c>
       <c r="O220" s="28" t="n">
-        <v>0.52325</v>
+        <v>0.522381</v>
       </c>
       <c r="P220" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q220" s="28" t="n">
-        <v>0.02325</v>
+        <v>-0.003685</v>
       </c>
       <c r="R220" s="26" t="n">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="S220" s="29" t="n">
         <v>1</v>
@@ -67698,7 +67698,7 @@
       <c r="AD220" s="24" t="n"/>
       <c r="AE220" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.13-3.98; raw selected-side p=0.5703, calibrated p=0.5233.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.13-3.98; raw selected-side p=0.5667, calibrated p=0.5224.</t>
         </is>
       </c>
       <c r="AF220" s="31" t="inlineStr">
@@ -67817,7 +67817,7 @@
       </c>
       <c r="BH220" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI220" s="24" t="inlineStr">
@@ -67829,16 +67829,16 @@
         <v>8.5</v>
       </c>
       <c r="BK220" s="26" t="n">
-        <v>100</v>
+        <v>-111</v>
       </c>
       <c r="BL220" s="27" t="n">
-        <v>2</v>
+        <v>1.900901</v>
       </c>
       <c r="BM220" s="28" t="n">
-        <v>0.5</v>
+        <v>0.526066</v>
       </c>
       <c r="BN220" s="28" t="n">
-        <v>0.497512</v>
+        <v>0.522388</v>
       </c>
       <c r="BO220" s="28" t="n"/>
       <c r="BP220" s="25" t="n"/>
@@ -67872,19 +67872,19 @@
       <c r="CR220" s="24" t="n"/>
       <c r="CS220" s="24" t="inlineStr">
         <is>
-          <t>True</t>
+          <t>False</t>
         </is>
       </c>
     </row>
     <row r="221" ht="36" customHeight="1">
       <c r="A221" s="24" t="inlineStr">
         <is>
-          <t>ba991f0b9ea64ab9</t>
+          <t>6c7fdfd427e540ad</t>
         </is>
       </c>
       <c r="B221" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C221" s="24" t="inlineStr">
@@ -67940,16 +67940,16 @@
         <v>0.635036</v>
       </c>
       <c r="O221" s="28" t="n">
-        <v>0.639346</v>
+        <v>0.639551</v>
       </c>
       <c r="P221" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q221" s="28" t="n">
-        <v>0.00431</v>
+        <v>0.004515</v>
       </c>
       <c r="R221" s="26" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S221" s="29" t="n">
         <v>1.75</v>
@@ -67975,7 +67975,7 @@
       <c r="AD221" s="24" t="n"/>
       <c r="AE221" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.38-4.11; raw selected-side p=0.7045, calibrated p=0.6393.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.38-4.11; raw selected-side p=0.7048, calibrated p=0.6396.</t>
         </is>
       </c>
       <c r="AF221" s="31" t="inlineStr">
@@ -68094,7 +68094,7 @@
       </c>
       <c r="BH221" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI221" s="24" t="inlineStr">
@@ -68156,12 +68156,12 @@
     <row r="222" ht="36" customHeight="1">
       <c r="A222" s="24" t="inlineStr">
         <is>
-          <t>f0a23255eaaa4207</t>
+          <t>fbf4b19abd124423</t>
         </is>
       </c>
       <c r="B222" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C222" s="24" t="inlineStr">
@@ -68208,25 +68208,25 @@
         </is>
       </c>
       <c r="L222" s="26" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="M222" s="27" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="N222" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.480769</v>
       </c>
       <c r="O222" s="28" t="n">
-        <v>0.51201</v>
+        <v>0.513637</v>
       </c>
       <c r="P222" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q222" s="28" t="n">
-        <v>0.038076</v>
+        <v>0.032868</v>
       </c>
       <c r="R222" s="26" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="S222" s="29" t="n">
         <v>1</v>
@@ -68252,7 +68252,7 @@
       <c r="AD222" s="24" t="n"/>
       <c r="AE222" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.38-4.11; raw selected-side p=0.5250, calibrated p=0.5120.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.38-4.11; raw selected-side p=0.5315, calibrated p=0.5136.</t>
         </is>
       </c>
       <c r="AF222" s="31" t="inlineStr">
@@ -68371,7 +68371,7 @@
       </c>
       <c r="BH222" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI222" s="24" t="inlineStr">
@@ -68383,16 +68383,16 @@
         <v>8.5</v>
       </c>
       <c r="BK222" s="26" t="n">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="BL222" s="27" t="n">
-        <v>2.11</v>
+        <v>2.08</v>
       </c>
       <c r="BM222" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.480769</v>
       </c>
       <c r="BN222" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.477612</v>
       </c>
       <c r="BO222" s="28" t="n"/>
       <c r="BP222" s="25" t="n"/>
@@ -68433,12 +68433,12 @@
     <row r="223" ht="36" customHeight="1">
       <c r="A223" s="24" t="inlineStr">
         <is>
-          <t>fa3e2c85412847c3</t>
+          <t>cb88912e18744f3e</t>
         </is>
       </c>
       <c r="B223" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C223" s="24" t="inlineStr">
@@ -68494,16 +68494,16 @@
         <v>0.640288</v>
       </c>
       <c r="O223" s="28" t="n">
-        <v>0.590354</v>
+        <v>0.586402</v>
       </c>
       <c r="P223" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q223" s="28" t="n">
-        <v>-0.049934</v>
+        <v>-0.053886</v>
       </c>
       <c r="R223" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S223" s="29" t="n">
         <v>1.25</v>
@@ -68529,7 +68529,7 @@
       <c r="AD223" s="24" t="n"/>
       <c r="AE223" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.27-4.68; raw selected-side p=0.6326, calibrated p=0.5904.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.27-4.68; raw selected-side p=0.6268, calibrated p=0.5864.</t>
         </is>
       </c>
       <c r="AF223" s="31" t="inlineStr">
@@ -68648,7 +68648,7 @@
       </c>
       <c r="BH223" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI223" s="24" t="inlineStr">
@@ -68710,12 +68710,12 @@
     <row r="224" ht="36" customHeight="1">
       <c r="A224" s="24" t="inlineStr">
         <is>
-          <t>38e7ec7e31dd40c3</t>
+          <t>f776c4b504a54715</t>
         </is>
       </c>
       <c r="B224" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C224" s="24" t="inlineStr">
@@ -68762,25 +68762,25 @@
         </is>
       </c>
       <c r="L224" s="26" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="M224" s="27" t="n">
-        <v>2.11</v>
+        <v>2.17</v>
       </c>
       <c r="N224" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.460829</v>
       </c>
       <c r="O224" s="28" t="n">
-        <v>0.527448</v>
+        <v>0.527398</v>
       </c>
       <c r="P224" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q224" s="28" t="n">
-        <v>0.053514</v>
+        <v>0.066569</v>
       </c>
       <c r="R224" s="26" t="n">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="S224" s="29" t="n">
         <v>1</v>
@@ -68806,7 +68806,7 @@
       <c r="AD224" s="24" t="n"/>
       <c r="AE224" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.27-4.68; raw selected-side p=0.5871, calibrated p=0.5274.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.27-4.68; raw selected-side p=0.5869, calibrated p=0.5274.</t>
         </is>
       </c>
       <c r="AF224" s="31" t="inlineStr">
@@ -68925,7 +68925,7 @@
       </c>
       <c r="BH224" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI224" s="24" t="inlineStr">
@@ -68937,16 +68937,16 @@
         <v>7.5</v>
       </c>
       <c r="BK224" s="26" t="n">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="BL224" s="27" t="n">
-        <v>2.11</v>
+        <v>2.17</v>
       </c>
       <c r="BM224" s="28" t="n">
-        <v>0.473934</v>
+        <v>0.460829</v>
       </c>
       <c r="BN224" s="28" t="n">
-        <v>0.472637</v>
+        <v>0.457711</v>
       </c>
       <c r="BO224" s="28" t="n"/>
       <c r="BP224" s="25" t="n"/>
@@ -68987,12 +68987,12 @@
     <row r="225" ht="36" customHeight="1">
       <c r="A225" s="24" t="inlineStr">
         <is>
-          <t>b58820a536ec4f82</t>
+          <t>7847dc728e3644d6</t>
         </is>
       </c>
       <c r="B225" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C225" s="24" t="inlineStr">
@@ -69039,25 +69039,25 @@
         </is>
       </c>
       <c r="L225" s="26" t="n">
-        <v>-174</v>
+        <v>-178</v>
       </c>
       <c r="M225" s="27" t="n">
-        <v>1.574713</v>
+        <v>1.561798</v>
       </c>
       <c r="N225" s="28" t="n">
-        <v>0.635036</v>
+        <v>0.640288</v>
       </c>
       <c r="O225" s="28" t="n">
-        <v>0.647353</v>
+        <v>0.648545</v>
       </c>
       <c r="P225" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q225" s="28" t="n">
-        <v>0.012317</v>
+        <v>0.008257</v>
       </c>
       <c r="R225" s="26" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="S225" s="29" t="n">
         <v>1.75</v>
@@ -69083,7 +69083,7 @@
       <c r="AD225" s="24" t="n"/>
       <c r="AE225" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.58-5.19; raw selected-side p=0.7163, calibrated p=0.6474.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.58-5.19; raw selected-side p=0.7180, calibrated p=0.6485.</t>
         </is>
       </c>
       <c r="AF225" s="31" t="inlineStr">
@@ -69202,7 +69202,7 @@
       </c>
       <c r="BH225" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI225" s="24" t="inlineStr">
@@ -69214,16 +69214,16 @@
         <v>1.5</v>
       </c>
       <c r="BK225" s="26" t="n">
-        <v>-174</v>
+        <v>-178</v>
       </c>
       <c r="BL225" s="27" t="n">
-        <v>1.574713</v>
+        <v>1.561798</v>
       </c>
       <c r="BM225" s="28" t="n">
-        <v>0.635036</v>
+        <v>0.640288</v>
       </c>
       <c r="BN225" s="28" t="n">
-        <v>0.631841</v>
+        <v>0.636816</v>
       </c>
       <c r="BO225" s="28" t="n"/>
       <c r="BP225" s="25" t="n"/>
@@ -69264,12 +69264,12 @@
     <row r="226" ht="36" customHeight="1">
       <c r="A226" s="24" t="inlineStr">
         <is>
-          <t>bd50730c4fab42bb</t>
+          <t>3a3a3a079e0b4ac3</t>
         </is>
       </c>
       <c r="B226" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C226" s="24" t="inlineStr">
@@ -69304,11 +69304,11 @@
       </c>
       <c r="I226" s="24" t="inlineStr">
         <is>
-          <t>under</t>
+          <t>over</t>
         </is>
       </c>
       <c r="J226" s="25" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="K226" s="24" t="inlineStr">
         <is>
@@ -69316,25 +69316,25 @@
         </is>
       </c>
       <c r="L226" s="26" t="n">
-        <v>-122</v>
+        <v>-111</v>
       </c>
       <c r="M226" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.900901</v>
       </c>
       <c r="N226" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.526066</v>
       </c>
       <c r="O226" s="28" t="n">
-        <v>0.51355</v>
+        <v>0.524778</v>
       </c>
       <c r="P226" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q226" s="28" t="n">
-        <v>-0.036</v>
+        <v>-0.001288</v>
       </c>
       <c r="R226" s="26" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="S226" s="29" t="n">
         <v>1</v>
@@ -69360,7 +69360,7 @@
       <c r="AD226" s="24" t="n"/>
       <c r="AE226" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.58-5.19; raw selected-side p=0.5312, calibrated p=0.5136.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.58-5.19; raw selected-side p=0.5764, calibrated p=0.5248.</t>
         </is>
       </c>
       <c r="AF226" s="31" t="inlineStr">
@@ -69479,7 +69479,7 @@
       </c>
       <c r="BH226" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI226" s="24" t="inlineStr">
@@ -69488,19 +69488,19 @@
         </is>
       </c>
       <c r="BJ226" s="25" t="n">
-        <v>9.5</v>
+        <v>8.5</v>
       </c>
       <c r="BK226" s="26" t="n">
-        <v>-122</v>
+        <v>-111</v>
       </c>
       <c r="BL226" s="27" t="n">
-        <v>1.819672</v>
+        <v>1.900901</v>
       </c>
       <c r="BM226" s="28" t="n">
-        <v>0.54955</v>
+        <v>0.526066</v>
       </c>
       <c r="BN226" s="28" t="n">
-        <v>0.547264</v>
+        <v>0.522388</v>
       </c>
       <c r="BO226" s="28" t="n"/>
       <c r="BP226" s="25" t="n"/>
@@ -69541,12 +69541,12 @@
     <row r="227" ht="36" customHeight="1">
       <c r="A227" s="24" t="inlineStr">
         <is>
-          <t>bcc44891645f4282</t>
+          <t>a7a64cb2e98c4d4c</t>
         </is>
       </c>
       <c r="B227" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C227" s="24" t="inlineStr">
@@ -69593,25 +69593,25 @@
         </is>
       </c>
       <c r="L227" s="26" t="n">
-        <v>-156</v>
+        <v>-153</v>
       </c>
       <c r="M227" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.653595</v>
       </c>
       <c r="N227" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.604743</v>
       </c>
       <c r="O227" s="28" t="n">
-        <v>0.631715</v>
+        <v>0.633554</v>
       </c>
       <c r="P227" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q227" s="28" t="n">
-        <v>0.02234</v>
+        <v>0.028811</v>
       </c>
       <c r="R227" s="26" t="n">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="S227" s="29" t="n">
         <v>1.5</v>
@@ -69637,7 +69637,7 @@
       <c r="AD227" s="24" t="n"/>
       <c r="AE227" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.87-4.56; raw selected-side p=0.6933, calibrated p=0.6317.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.87-4.56; raw selected-side p=0.6960, calibrated p=0.6336.</t>
         </is>
       </c>
       <c r="AF227" s="31" t="inlineStr">
@@ -69756,7 +69756,7 @@
       </c>
       <c r="BH227" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI227" s="24" t="inlineStr">
@@ -69768,16 +69768,16 @@
         <v>1.5</v>
       </c>
       <c r="BK227" s="26" t="n">
-        <v>-156</v>
+        <v>-153</v>
       </c>
       <c r="BL227" s="27" t="n">
-        <v>1.641026</v>
+        <v>1.653595</v>
       </c>
       <c r="BM227" s="28" t="n">
-        <v>0.609375</v>
+        <v>0.604743</v>
       </c>
       <c r="BN227" s="28" t="n">
-        <v>0.606965</v>
+        <v>0.60199</v>
       </c>
       <c r="BO227" s="28" t="n"/>
       <c r="BP227" s="25" t="n"/>
@@ -69818,12 +69818,12 @@
     <row r="228" ht="36" customHeight="1">
       <c r="A228" s="24" t="inlineStr">
         <is>
-          <t>ad2ee23048d3470b</t>
+          <t>4cff1e5dcda04b4c</t>
         </is>
       </c>
       <c r="B228" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C228" s="24" t="inlineStr">
@@ -69870,25 +69870,25 @@
         </is>
       </c>
       <c r="L228" s="26" t="n">
-        <v>-113</v>
+        <v>-102</v>
       </c>
       <c r="M228" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.980392</v>
       </c>
       <c r="N228" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.50495</v>
       </c>
       <c r="O228" s="28" t="n">
-        <v>0.537198</v>
+        <v>0.537173</v>
       </c>
       <c r="P228" s="28" t="n">
         <v>0.042131</v>
       </c>
       <c r="Q228" s="28" t="n">
-        <v>0.006682</v>
+        <v>0.032223</v>
       </c>
       <c r="R228" s="26" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="S228" s="29" t="n">
         <v>1</v>
@@ -69914,7 +69914,7 @@
       <c r="AD228" s="24" t="n"/>
       <c r="AE228" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.87-4.56; raw selected-side p=0.6264, calibrated p=0.5372.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.87-4.56; raw selected-side p=0.6263, calibrated p=0.5372.</t>
         </is>
       </c>
       <c r="AF228" s="31" t="inlineStr">
@@ -70033,7 +70033,7 @@
       </c>
       <c r="BH228" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI228" s="24" t="inlineStr">
@@ -70045,16 +70045,16 @@
         <v>7.5</v>
       </c>
       <c r="BK228" s="26" t="n">
-        <v>-113</v>
+        <v>-102</v>
       </c>
       <c r="BL228" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.980392</v>
       </c>
       <c r="BM228" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.50495</v>
       </c>
       <c r="BN228" s="28" t="n">
-        <v>0.527363</v>
+        <v>0.502488</v>
       </c>
       <c r="BO228" s="28" t="n"/>
       <c r="BP228" s="25" t="n"/>
@@ -70095,12 +70095,12 @@
     <row r="229" ht="36" customHeight="1">
       <c r="A229" s="24" t="inlineStr">
         <is>
-          <t>d1c934f6d02e4c3f</t>
+          <t>3b8fce910aa54bd0</t>
         </is>
       </c>
       <c r="B229" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C229" s="24" t="inlineStr">
@@ -70147,25 +70147,25 @@
         </is>
       </c>
       <c r="L229" s="26" t="n">
-        <v>-150</v>
+        <v>-141</v>
       </c>
       <c r="M229" s="27" t="n">
-        <v>1.666667</v>
+        <v>1.70922</v>
       </c>
       <c r="N229" s="28" t="n">
-        <v>0.6</v>
+        <v>0.585062</v>
       </c>
       <c r="O229" s="28" t="n">
-        <v>0.580303</v>
+        <v>0.5781230000000001</v>
       </c>
       <c r="P229" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q229" s="28" t="n">
-        <v>-0.019697</v>
+        <v>-0.006939</v>
       </c>
       <c r="R229" s="26" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="S229" s="29" t="n">
         <v>1.25</v>
@@ -70191,7 +70191,7 @@
       <c r="AD229" s="24" t="n"/>
       <c r="AE229" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Margin: Trend Engine projected 4.83-4.33; raw selected-side p=0.6179, calibrated p=0.5803.</t>
+          <t>Measured Edge Margin: Trend Engine projected 4.83-4.33; raw selected-side p=0.6147, calibrated p=0.5781.</t>
         </is>
       </c>
       <c r="AF229" s="31" t="inlineStr">
@@ -70310,7 +70310,7 @@
       </c>
       <c r="BH229" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI229" s="24" t="inlineStr">
@@ -70322,16 +70322,16 @@
         <v>1.5</v>
       </c>
       <c r="BK229" s="26" t="n">
-        <v>-150</v>
+        <v>-141</v>
       </c>
       <c r="BL229" s="27" t="n">
-        <v>1.666667</v>
+        <v>1.70922</v>
       </c>
       <c r="BM229" s="28" t="n">
-        <v>0.6</v>
+        <v>0.585062</v>
       </c>
       <c r="BN229" s="28" t="n">
-        <v>0.597015</v>
+        <v>0.58209</v>
       </c>
       <c r="BO229" s="28" t="n"/>
       <c r="BP229" s="25" t="n"/>
@@ -70372,12 +70372,12 @@
     <row r="230" ht="36" customHeight="1">
       <c r="A230" s="24" t="inlineStr">
         <is>
-          <t>2cf016d817bc4758</t>
+          <t>1c707594d7d54d7c</t>
         </is>
       </c>
       <c r="B230" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="C230" s="24" t="inlineStr">
@@ -70424,25 +70424,25 @@
         </is>
       </c>
       <c r="L230" s="26" t="n">
-        <v>-113</v>
+        <v>-120</v>
       </c>
       <c r="M230" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.833333</v>
       </c>
       <c r="N230" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.545455</v>
       </c>
       <c r="O230" s="28" t="n">
-        <v>0.527374</v>
+        <v>0.526914</v>
       </c>
       <c r="P230" s="28" t="n">
         <v>0.05172</v>
       </c>
       <c r="Q230" s="28" t="n">
-        <v>-0.003142</v>
+        <v>-0.018541</v>
       </c>
       <c r="R230" s="26" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="S230" s="29" t="n">
         <v>1</v>
@@ -70468,7 +70468,7 @@
       <c r="AD230" s="24" t="n"/>
       <c r="AE230" s="31" t="inlineStr">
         <is>
-          <t>Measured Edge Totals: Trend Engine projected 4.83-4.33; raw selected-side p=0.5868, calibrated p=0.5274.</t>
+          <t>Measured Edge Totals: Trend Engine projected 4.83-4.33; raw selected-side p=0.5850, calibrated p=0.5269.</t>
         </is>
       </c>
       <c r="AF230" s="31" t="inlineStr">
@@ -70587,7 +70587,7 @@
       </c>
       <c r="BH230" s="24" t="inlineStr">
         <is>
-          <t>2026-08-05T04:36:16.771749Z</t>
+          <t>2026-08-05T13:54:46.877508Z</t>
         </is>
       </c>
       <c r="BI230" s="24" t="inlineStr">
@@ -70599,16 +70599,16 @@
         <v>9.5</v>
       </c>
       <c r="BK230" s="26" t="n">
-        <v>-113</v>
+        <v>-120</v>
       </c>
       <c r="BL230" s="27" t="n">
-        <v>1.884956</v>
+        <v>1.833333</v>
       </c>
       <c r="BM230" s="28" t="n">
-        <v>0.530516</v>
+        <v>0.545455</v>
       </c>
       <c r="BN230" s="28" t="n">
-        <v>0.527363</v>
+        <v>0.542289</v>
       </c>
       <c r="BO230" s="28" t="n"/>
       <c r="BP230" s="25" t="n"/>

</xml_diff>